<commit_message>
feat: support shared tutorial players and config workflows
</commit_message>
<xml_diff>
--- a/configs/Datas/#Player.xlsx
+++ b/configs/Datas/#Player.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="173">
   <si>
     <t>##var</t>
   </si>
@@ -208,7 +208,7 @@
     <t>player_apex</t>
   </si>
   <si>
-    <t>豆豆</t>
+    <t>apex</t>
   </si>
   <si>
     <t>team_vitality</t>
@@ -232,7 +232,7 @@
     <t>player_flamez</t>
   </si>
   <si>
-    <t>火仔</t>
+    <t>flameZ</t>
   </si>
   <si>
     <t>Anchor</t>
@@ -250,7 +250,7 @@
     <t>player_zywoo</t>
   </si>
   <si>
-    <t>载物</t>
+    <t>ZyWOo</t>
   </si>
   <si>
     <t>DK</t>
@@ -271,7 +271,7 @@
     <t>player_mezii</t>
   </si>
   <si>
-    <t>妹子</t>
+    <t>mezii</t>
   </si>
   <si>
     <t>UA</t>
@@ -289,7 +289,7 @@
     <t>player_ropz</t>
   </si>
   <si>
-    <t>车主</t>
+    <t>ropz</t>
   </si>
   <si>
     <t>FI</t>
@@ -310,7 +310,7 @@
     <t>player_kyousuke</t>
   </si>
   <si>
-    <t>京介</t>
+    <t>kyousuke</t>
   </si>
   <si>
     <t>team_falcons</t>
@@ -325,13 +325,13 @@
     <t>portraits/player_kyousuke.jpg</t>
   </si>
   <si>
-    <t>player-cards/kyousuke.png</t>
+    <t>player-cards/kyousuke2.png</t>
   </si>
   <si>
     <t>player_kyxsan</t>
   </si>
   <si>
-    <t>K3</t>
+    <t>karrigan</t>
   </si>
   <si>
     <t>NO</t>
@@ -340,10 +340,13 @@
     <t>portraits/player_kyxsan.jpg</t>
   </si>
   <si>
+    <t>player-cards/karrigan.png</t>
+  </si>
+  <si>
     <t>player_monesy</t>
   </si>
   <si>
-    <t>孩神</t>
+    <t>m0NESY</t>
   </si>
   <si>
     <t>SE</t>
@@ -358,10 +361,10 @@
     <t>player_niko</t>
   </si>
   <si>
-    <t>老尼</t>
-  </si>
-  <si>
-    <t>AWPer,IGL</t>
+    <t>NiKo</t>
+  </si>
+  <si>
+    <t>Rifler</t>
   </si>
   <si>
     <t>portraits/player_niko.jpg</t>
@@ -373,7 +376,7 @@
     <t>player_teses</t>
   </si>
   <si>
-    <t>龙哥</t>
+    <t>TeSeS</t>
   </si>
   <si>
     <t>RU</t>
@@ -382,6 +385,9 @@
     <t>IGL,AWPer</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
     <t>portraits/player_teses.jpg</t>
   </si>
   <si>
@@ -421,19 +427,19 @@
     <t>player_chopper</t>
   </si>
   <si>
-    <t>chopper</t>
+    <t>tn1r</t>
   </si>
   <si>
     <t>portraits/player_chopper.jpg</t>
   </si>
   <si>
+    <t>player-cards/tn1r.png</t>
+  </si>
+  <si>
     <t>player_zont1x</t>
   </si>
   <si>
     <t>zont1x</t>
-  </si>
-  <si>
-    <t>Rifler</t>
   </si>
   <si>
     <t>portraits/player_zont1x.jpg</t>
@@ -1219,16 +1225,16 @@
         <v>71</v>
       </c>
       <c r="Y5" s="1">
-        <v>0.251924</v>
+        <v>0.29231</v>
       </c>
       <c r="Z5" s="1">
         <v>0.097308</v>
       </c>
       <c r="AA5" s="1">
-        <v>0.524998</v>
+        <v>0.470189</v>
       </c>
       <c r="AB5" s="1">
-        <v>0.489998</v>
+        <v>0.438843</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
@@ -1302,16 +1308,16 @@
         <v>77</v>
       </c>
       <c r="Y6" s="1">
-        <v>0.2</v>
+        <v>0.260579</v>
       </c>
       <c r="Z6" s="1">
-        <v>0.08</v>
+        <v>0.112693</v>
       </c>
       <c r="AA6" s="1">
-        <v>0.6</v>
+        <v>0.435572</v>
       </c>
       <c r="AB6" s="1">
-        <v>0.56</v>
+        <v>0.406534</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
@@ -1385,16 +1391,16 @@
         <v>84</v>
       </c>
       <c r="Y7" s="1">
-        <v>0.2</v>
+        <v>0.246155</v>
       </c>
       <c r="Z7" s="1">
-        <v>0.08</v>
+        <v>0.105001</v>
       </c>
       <c r="AA7" s="1">
-        <v>0.6</v>
+        <v>0.484612</v>
       </c>
       <c r="AB7" s="1">
-        <v>0.56</v>
+        <v>0.452304</v>
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
@@ -1468,16 +1474,16 @@
         <v>90</v>
       </c>
       <c r="Y8" s="1">
-        <v>0.2</v>
+        <v>0.260579</v>
       </c>
       <c r="Z8" s="1">
-        <v>0.08</v>
+        <v>0.087693</v>
       </c>
       <c r="AA8" s="1">
-        <v>0.6</v>
+        <v>0.473073</v>
       </c>
       <c r="AB8" s="1">
-        <v>0.56</v>
+        <v>0.441535</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
@@ -1551,16 +1557,16 @@
         <v>97</v>
       </c>
       <c r="Y9" s="1">
-        <v>0.2</v>
+        <v>0.237501</v>
       </c>
       <c r="Z9" s="1">
-        <v>0.08</v>
+        <v>0.091538</v>
       </c>
       <c r="AA9" s="1">
-        <v>0.6</v>
+        <v>0.461534</v>
       </c>
       <c r="AB9" s="1">
-        <v>0.56</v>
+        <v>0.430766</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
@@ -1634,16 +1640,16 @@
         <v>104</v>
       </c>
       <c r="Y10" s="1">
-        <v>0.2</v>
+        <v>0.262508</v>
       </c>
       <c r="Z10" s="1">
-        <v>0.08</v>
+        <v>0.06154</v>
       </c>
       <c r="AA10" s="1">
-        <v>0.6</v>
+        <v>0.524024</v>
       </c>
       <c r="AB10" s="1">
-        <v>0.56</v>
+        <v>0.489089</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
@@ -1713,31 +1719,34 @@
       <c r="W11" t="s">
         <v>108</v>
       </c>
+      <c r="X11" t="s">
+        <v>109</v>
+      </c>
       <c r="Y11" s="1">
-        <v>0</v>
+        <v>0.233661</v>
       </c>
       <c r="Z11" s="1">
-        <v>0</v>
+        <v>0.096797</v>
       </c>
       <c r="AA11" s="1">
-        <v>0</v>
+        <v>0.512485</v>
       </c>
       <c r="AB11" s="1">
-        <v>0</v>
+        <v>0.47832</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D12" t="s">
         <v>100</v>
       </c>
       <c r="E12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F12">
         <v>95</v>
@@ -1791,30 +1800,30 @@
         <v>69</v>
       </c>
       <c r="W12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="X12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Y12" s="1">
-        <v>0.2</v>
+        <v>0.217308</v>
       </c>
       <c r="Z12" s="1">
-        <v>0.08</v>
+        <v>0.078077</v>
       </c>
       <c r="AA12" s="1">
-        <v>0.6</v>
+        <v>0.559614</v>
       </c>
       <c r="AB12" s="1">
-        <v>0.56</v>
+        <v>0.522307</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
         <v>100</v>
@@ -1868,16 +1877,16 @@
         <v>80</v>
       </c>
       <c r="U13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="V13" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="W13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Y13" s="1">
         <v>0.217308</v>
@@ -1894,16 +1903,16 @@
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D14" t="s">
         <v>100</v>
       </c>
       <c r="E14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F14">
         <v>90</v>
@@ -1951,42 +1960,42 @@
         <v>92</v>
       </c>
       <c r="U14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="V14" t="s">
-        <v>82</v>
+        <v>124</v>
       </c>
       <c r="W14" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="X14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="Y14" s="1">
         <v>0.2</v>
       </c>
       <c r="Z14" s="1">
-        <v>0.08</v>
+        <v>0.068461</v>
       </c>
       <c r="AA14" s="1">
-        <v>0.6</v>
+        <v>0.545191</v>
       </c>
       <c r="AB14" s="1">
-        <v>0.56</v>
+        <v>0.508845</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C15" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F15">
         <v>94</v>
@@ -2034,42 +2043,42 @@
         <v>83</v>
       </c>
       <c r="U15" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="V15" t="s">
         <v>75</v>
       </c>
       <c r="W15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="X15" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="Y15" s="1">
-        <v>0.2</v>
+        <v>0.257695</v>
       </c>
       <c r="Z15" s="1">
-        <v>0.08</v>
+        <v>0.081923</v>
       </c>
       <c r="AA15" s="1">
-        <v>0.6</v>
+        <v>0.40961</v>
       </c>
       <c r="AB15" s="1">
-        <v>0.56</v>
+        <v>0.382303</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C16" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F16">
         <v>74</v>
@@ -2123,36 +2132,36 @@
         <v>75</v>
       </c>
       <c r="W16" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="X16" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="Y16" s="1">
-        <v>0.2</v>
+        <v>0.231732</v>
       </c>
       <c r="Z16" s="1">
-        <v>0.08</v>
+        <v>0.072307</v>
       </c>
       <c r="AA16" s="1">
-        <v>0.6</v>
+        <v>0.421148</v>
       </c>
       <c r="AB16" s="1">
-        <v>0.56</v>
+        <v>0.393072</v>
       </c>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C17" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D17" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E17" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F17">
         <v>72</v>
@@ -2206,30 +2215,33 @@
         <v>69</v>
       </c>
       <c r="W17" t="s">
-        <v>137</v>
+        <v>139</v>
+      </c>
+      <c r="X17" t="s">
+        <v>140</v>
       </c>
       <c r="Y17" s="1">
-        <v>0</v>
+        <v>0.265393</v>
       </c>
       <c r="Z17" s="1">
-        <v>0</v>
+        <v>0.090258</v>
       </c>
       <c r="AA17" s="1">
-        <v>0</v>
+        <v>0.425944</v>
       </c>
       <c r="AB17" s="1">
-        <v>0</v>
+        <v>0.397548</v>
       </c>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D18" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E18" t="s">
         <v>87</v>
@@ -2280,42 +2292,42 @@
         <v>90</v>
       </c>
       <c r="U18" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="V18" t="s">
         <v>69</v>
       </c>
       <c r="W18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="X18" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Y18" s="1">
-        <v>0.2</v>
+        <v>0.286541</v>
       </c>
       <c r="Z18" s="1">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="AA18" s="1">
-        <v>0.6</v>
+        <v>0.389417</v>
       </c>
       <c r="AB18" s="1">
-        <v>0.56</v>
+        <v>0.363456</v>
       </c>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C19" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D19" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F19">
         <v>78</v>
@@ -2363,39 +2375,39 @@
         <v>91</v>
       </c>
       <c r="U19" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="V19" t="s">
         <v>69</v>
       </c>
       <c r="W19" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="X19" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Y19" s="1">
-        <v>0.2</v>
+        <v>0.277887</v>
       </c>
       <c r="Z19" s="1">
-        <v>0.08</v>
+        <v>0.07</v>
       </c>
       <c r="AA19" s="1">
-        <v>0.6</v>
+        <v>0.377878</v>
       </c>
       <c r="AB19" s="1">
-        <v>0.56</v>
+        <v>0.352686</v>
       </c>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C20" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D20" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E20" t="s">
         <v>87</v>
@@ -2446,39 +2458,39 @@
         <v>90</v>
       </c>
       <c r="U20" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="V20" t="s">
         <v>75</v>
       </c>
       <c r="W20" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="X20" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="Y20" s="1">
-        <v>0.2</v>
+        <v>0.286541</v>
       </c>
       <c r="Z20" s="1">
-        <v>0.08</v>
+        <v>0.06923</v>
       </c>
       <c r="AA20" s="1">
-        <v>0.6</v>
+        <v>0.380763</v>
       </c>
       <c r="AB20" s="1">
-        <v>0.56</v>
+        <v>0.355379</v>
       </c>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D21" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E21" t="s">
         <v>87</v>
@@ -2535,36 +2547,36 @@
         <v>75</v>
       </c>
       <c r="W21" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="X21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="Y21" s="1">
-        <v>0.2</v>
+        <v>0.251925</v>
       </c>
       <c r="Z21" s="1">
-        <v>0.08</v>
+        <v>0.082308</v>
       </c>
       <c r="AA21" s="1">
-        <v>0.6</v>
+        <v>0.389417</v>
       </c>
       <c r="AB21" s="1">
-        <v>0.56</v>
+        <v>0.363456</v>
       </c>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C22" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D22" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E22" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F22">
         <v>91</v>
@@ -2612,39 +2624,39 @@
         <v>82</v>
       </c>
       <c r="U22" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="V22" t="s">
         <v>69</v>
       </c>
       <c r="W22" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="X22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="Y22" s="1">
-        <v>0.2</v>
+        <v>0.277887</v>
       </c>
       <c r="Z22" s="1">
-        <v>0.08</v>
+        <v>0.066922</v>
       </c>
       <c r="AA22" s="1">
-        <v>0.6</v>
+        <v>0.389417</v>
       </c>
       <c r="AB22" s="1">
-        <v>0.56</v>
+        <v>0.363456</v>
       </c>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C23" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D23" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E23" t="s">
         <v>93</v>
@@ -2701,36 +2713,36 @@
         <v>69</v>
       </c>
       <c r="W23" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="X23" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="Y23" s="1">
-        <v>0.2</v>
+        <v>0.257694</v>
       </c>
       <c r="Z23" s="1">
-        <v>0.08</v>
+        <v>0.076154</v>
       </c>
       <c r="AA23" s="1">
-        <v>0.6</v>
+        <v>0.400956</v>
       </c>
       <c r="AB23" s="1">
-        <v>0.56</v>
+        <v>0.374225</v>
       </c>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C24" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D24" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E24" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F24">
         <v>88</v>
@@ -2778,28 +2790,28 @@
         <v>80</v>
       </c>
       <c r="U24" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="V24" t="s">
         <v>69</v>
       </c>
       <c r="W24" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="X24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="Y24" s="1">
-        <v>0.2</v>
+        <v>0.292311</v>
       </c>
       <c r="Z24" s="1">
-        <v>0.08</v>
+        <v>0.090385</v>
       </c>
       <c r="AA24" s="1">
-        <v>0.6</v>
+        <v>0.395186</v>
       </c>
       <c r="AB24" s="1">
-        <v>0.56</v>
+        <v>0.36884</v>
       </c>
     </row>
   </sheetData>

</xml_diff>